<commit_message>
Superintendent-pay: remove shared/joint framing of the Andover-Scotland contracts (per Val); rebuild
</commit_message>
<xml_diff>
--- a/reports/aes/superintendent-pay/contracts.xlsx
+++ b/reports/aes/superintendent-pay/contracts.xlsx
@@ -227,135 +227,135 @@
     <t>Donna P. Leake</t>
   </si>
   <si>
+    <t>2021-07-01</t>
+  </si>
+  <si>
+    <t>eastford/MANUAL__Leake_Eastford_2026-27_Amendment.pdf</t>
+  </si>
+  <si>
+    <t>Hampton</t>
+  </si>
+  <si>
+    <t>Andrew Skarzynski</t>
+  </si>
+  <si>
+    <t>hampton/CONTRACT_A.Skarzynski_25-28.pdf</t>
+  </si>
+  <si>
+    <t>Hebron</t>
+  </si>
+  <si>
+    <t>Dr. Thomas Baird</t>
+  </si>
+  <si>
+    <t>hebron/KNOWN__GetFile_ashx.pdf</t>
+  </si>
+  <si>
+    <t>Lisbon</t>
+  </si>
+  <si>
+    <t>Sally A. Keating</t>
+  </si>
+  <si>
+    <t>lisbon/score150__d2__Superintendent-Contract-2026-2028.pdf</t>
+  </si>
+  <si>
+    <t>New Hartford</t>
+  </si>
+  <si>
+    <t>Jeffrey F. Sousa</t>
+  </si>
+  <si>
+    <t>new-hartford/Sousa_NewHartford_K6_2023-2026.pdf</t>
+  </si>
+  <si>
+    <t>Norfolk</t>
+  </si>
+  <si>
+    <t>Mary Beth Iacobelli</t>
+  </si>
+  <si>
+    <t>2022-07-01</t>
+  </si>
+  <si>
+    <t>2025-06-30</t>
+  </si>
+  <si>
+    <t>norfolk/score220__d2__BOE-Superintendent-Contract-2022-2025_pdf.pdf</t>
+  </si>
+  <si>
+    <t>Preston</t>
+  </si>
+  <si>
+    <t>Dr. Roy Seitsinger</t>
+  </si>
+  <si>
+    <t>K-8 (assumed)</t>
+  </si>
+  <si>
+    <t>preston/score170__d2__4775.pdf</t>
+  </si>
+  <si>
+    <t>Redding</t>
+  </si>
+  <si>
+    <t>Voluntown</t>
+  </si>
+  <si>
+    <t>Scott Feder</t>
+  </si>
+  <si>
+    <t>voluntown/KNOWN__Superintendent-PDF.pdf</t>
+  </si>
+  <si>
+    <t>West Willington</t>
+  </si>
+  <si>
+    <t>Philip 'Phil' Stevens</t>
+  </si>
+  <si>
+    <t>2023-24</t>
+  </si>
+  <si>
+    <t>stale</t>
+  </si>
+  <si>
+    <t>west-willington/score150__d2__superintendent_contract_2022-2025pdf-PDF.pdf</t>
+  </si>
+  <si>
+    <t>Chaplin</t>
+  </si>
+  <si>
+    <t>K-12 (Region 11 + Chaplin)</t>
+  </si>
+  <si>
+    <t>2024-05-11</t>
+  </si>
+  <si>
+    <t>chaplin/score150__d2__superintendent_contract_2024-2027_pdf.pdf</t>
+  </si>
+  <si>
+    <t>Columbia</t>
+  </si>
+  <si>
+    <t>Barbara Wilson</t>
+  </si>
+  <si>
+    <t>2024-02-01</t>
+  </si>
+  <si>
+    <t>columbia/Wilson_Columbia_2024-2028.pdf</t>
+  </si>
+  <si>
+    <t>Scotland</t>
+  </si>
+  <si>
     <t>2021-22</t>
   </si>
   <si>
-    <t>2021-07-01</t>
-  </si>
-  <si>
     <t>2024-06-30</t>
   </si>
   <si>
-    <t>stale</t>
-  </si>
-  <si>
-    <t>eastford/KNOWN__Superintendent-Contract-2022_pdf.pdf</t>
-  </si>
-  <si>
-    <t>Hampton</t>
-  </si>
-  <si>
-    <t>Andrew Skarzynski</t>
-  </si>
-  <si>
-    <t>hampton/CONTRACT_A.Skarzynski_25-28.pdf</t>
-  </si>
-  <si>
-    <t>Hebron</t>
-  </si>
-  <si>
-    <t>Dr. Thomas Baird</t>
-  </si>
-  <si>
-    <t>hebron/KNOWN__GetFile_ashx.pdf</t>
-  </si>
-  <si>
-    <t>Lisbon</t>
-  </si>
-  <si>
-    <t>Sally A. Keating</t>
-  </si>
-  <si>
-    <t>lisbon/score150__d2__Superintendent-Contract-2026-2028.pdf</t>
-  </si>
-  <si>
-    <t>New Hartford</t>
-  </si>
-  <si>
-    <t>Jeffrey F. Sousa</t>
-  </si>
-  <si>
-    <t>new-hartford/Sousa_NewHartford_K6_2023-2026.pdf</t>
-  </si>
-  <si>
-    <t>Norfolk</t>
-  </si>
-  <si>
-    <t>Mary Beth Iacobelli</t>
-  </si>
-  <si>
-    <t>2022-07-01</t>
-  </si>
-  <si>
-    <t>2025-06-30</t>
-  </si>
-  <si>
-    <t>norfolk/score220__d2__BOE-Superintendent-Contract-2022-2025_pdf.pdf</t>
-  </si>
-  <si>
-    <t>Preston</t>
-  </si>
-  <si>
-    <t>Dr. Roy Seitsinger</t>
-  </si>
-  <si>
-    <t>K-8 (assumed)</t>
-  </si>
-  <si>
-    <t>preston/score170__d2__4775.pdf</t>
-  </si>
-  <si>
-    <t>Redding</t>
-  </si>
-  <si>
-    <t>Voluntown</t>
-  </si>
-  <si>
-    <t>Scott Feder</t>
-  </si>
-  <si>
-    <t>voluntown/KNOWN__Superintendent-PDF.pdf</t>
-  </si>
-  <si>
-    <t>West Willington</t>
-  </si>
-  <si>
-    <t>Philip 'Phil' Stevens</t>
-  </si>
-  <si>
-    <t>2023-24</t>
-  </si>
-  <si>
-    <t>west-willington/score150__d2__superintendent_contract_2022-2025pdf-PDF.pdf</t>
-  </si>
-  <si>
-    <t>Chaplin</t>
-  </si>
-  <si>
-    <t>K-12 (Region 11 + Chaplin)</t>
-  </si>
-  <si>
-    <t>2024-05-11</t>
-  </si>
-  <si>
-    <t>chaplin/score150__d2__superintendent_contract_2024-2027_pdf.pdf</t>
-  </si>
-  <si>
-    <t>Columbia</t>
-  </si>
-  <si>
-    <t>Barbara Wilson</t>
-  </si>
-  <si>
-    <t>2024-02-01</t>
-  </si>
-  <si>
-    <t>columbia/Wilson_Columbia_2024-2028.pdf</t>
-  </si>
-  <si>
-    <t>Scotland</t>
-  </si>
-  <si>
     <t>scotland/KNOWN__Bruneau_Scotland_2021-2024.pdf</t>
   </si>
   <si>
@@ -614,6 +614,9 @@
     <t>andover</t>
   </si>
   <si>
+    <t>eastford</t>
+  </si>
+  <si>
     <t>chaplin</t>
   </si>
   <si>
@@ -627,9 +630,6 @@
   </si>
   <si>
     <t>west-willington</t>
-  </si>
-  <si>
-    <t>eastford</t>
   </si>
   <si>
     <t>scotland</t>
@@ -1758,22 +1758,22 @@
         <v>22</v>
       </c>
       <c r="D13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" t="s">
-        <v>72</v>
-      </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="G13">
-        <v>0.392</v>
+        <v>0.4</v>
       </c>
       <c r="H13">
-        <v>0.392</v>
+        <v>0.4</v>
       </c>
       <c r="I13" s="1">
-        <v>57571</v>
+        <v>63478</v>
       </c>
       <c r="J13" s="1">
         <v>0</v>
@@ -1789,30 +1789,30 @@
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>57571</v>
+        <v>63478</v>
       </c>
       <c r="P13" s="1">
-        <v>146866</v>
+        <v>158695</v>
       </c>
       <c r="Q13" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="R13" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="S13" t="s">
         <v>28</v>
       </c>
       <c r="T13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1862,15 +1862,15 @@
         <v>28</v>
       </c>
       <c r="T14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
         <v>22</v>
@@ -1918,15 +1918,15 @@
         <v>28</v>
       </c>
       <c r="T15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C16" t="s">
         <v>44</v>
@@ -1978,15 +1978,15 @@
         <v>28</v>
       </c>
       <c r="T16" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C17" t="s">
         <v>22</v>
@@ -2038,15 +2038,15 @@
         <v>28</v>
       </c>
       <c r="T17" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
         <v>22</v>
@@ -2055,10 +2055,10 @@
         <v>63</v>
       </c>
       <c r="E18" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G18">
         <v>0.4</v>
@@ -2098,18 +2098,18 @@
         <v>28</v>
       </c>
       <c r="T18" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B19" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
         <v>23</v>
@@ -2156,12 +2156,12 @@
         <v>28</v>
       </c>
       <c r="T19" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B20" t="s">
         <v>66</v>
@@ -2221,13 +2221,13 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -2274,21 +2274,21 @@
         <v>28</v>
       </c>
       <c r="T21" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D22" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
         <v>24</v>
@@ -2328,30 +2328,30 @@
         <v>34</v>
       </c>
       <c r="R22" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="S22" t="s">
         <v>28</v>
       </c>
       <c r="T22" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" t="s">
         <v>105</v>
-      </c>
-      <c r="B23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C23" t="s">
-        <v>106</v>
-      </c>
-      <c r="D23" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" t="s">
-        <v>107</v>
       </c>
       <c r="F23" t="s">
         <v>49</v>
@@ -2392,15 +2392,15 @@
         <v>57</v>
       </c>
       <c r="T23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C24" t="s">
         <v>22</v>
@@ -2409,7 +2409,7 @@
         <v>23</v>
       </c>
       <c r="E24" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F24" t="s">
         <v>40</v>
@@ -2450,12 +2450,12 @@
         <v>28</v>
       </c>
       <c r="T24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B25" t="s">
         <v>21</v>
@@ -2464,13 +2464,13 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
+        <v>112</v>
+      </c>
+      <c r="E25" t="s">
         <v>71</v>
       </c>
-      <c r="E25" t="s">
-        <v>72</v>
-      </c>
       <c r="F25" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -2502,7 +2502,7 @@
         <v>34</v>
       </c>
       <c r="R25" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="S25" t="s">
         <v>28</v>
@@ -2818,7 +2818,7 @@
         <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E31" t="s">
         <v>24</v>
@@ -2852,7 +2852,7 @@
         <v>34</v>
       </c>
       <c r="R31" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="S31" t="s">
         <v>28</v>
@@ -4089,13 +4089,13 @@
         <v>181</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
         <v>45</v>
@@ -4128,7 +4128,7 @@
         <v>223736</v>
       </c>
       <c r="Q9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -4236,16 +4236,16 @@
         <v>184</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" t="s">
         <v>109</v>
-      </c>
-      <c r="E12" t="s">
-        <v>111</v>
       </c>
       <c r="F12" t="s">
         <v>40</v>
@@ -4277,7 +4277,7 @@
         <v>202400</v>
       </c>
       <c r="Q12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
@@ -4285,13 +4285,13 @@
         <v>185</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D13" t="s">
         <v>95</v>
-      </c>
-      <c r="D13" t="s">
-        <v>98</v>
       </c>
       <c r="E13" t="s">
         <v>45</v>
@@ -4326,7 +4326,7 @@
         <v>200000</v>
       </c>
       <c r="Q13" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
@@ -4483,13 +4483,13 @@
         <v>189</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C17" t="s">
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E17" t="s">
         <v>24</v>
@@ -4526,7 +4526,7 @@
         <v>193250</v>
       </c>
       <c r="Q17" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -4779,13 +4779,13 @@
         <v>195</v>
       </c>
       <c r="B23" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D23" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E23" t="s">
         <v>45</v>
@@ -4820,7 +4820,7 @@
         <v>179307</v>
       </c>
       <c r="Q23" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
@@ -4828,13 +4828,13 @@
         <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C24" t="s">
         <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E24" t="s">
         <v>45</v>
@@ -4869,7 +4869,7 @@
         <v>179167</v>
       </c>
       <c r="Q24" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -4926,19 +4926,19 @@
         <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
         <v>22</v>
       </c>
       <c r="D26" t="s">
+        <v>85</v>
+      </c>
+      <c r="E26" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26" t="s">
         <v>88</v>
-      </c>
-      <c r="E26" t="s">
-        <v>90</v>
-      </c>
-      <c r="F26" t="s">
-        <v>91</v>
       </c>
       <c r="G26" t="s">
         <v>63</v>
@@ -4969,7 +4969,7 @@
         <v>173750</v>
       </c>
       <c r="Q26" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
@@ -5026,16 +5026,16 @@
         <v>200</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>106</v>
+        <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="E28" t="s">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="F28" t="s">
         <v>49</v>
@@ -5047,27 +5047,29 @@
         <v>27</v>
       </c>
       <c r="I28" s="1">
-        <v>136750</v>
+        <v>63478</v>
       </c>
       <c r="J28" s="1">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="K28" s="1">
         <v>0</v>
       </c>
-      <c r="L28" s="1"/>
+      <c r="L28" s="1">
+        <v>0</v>
+      </c>
       <c r="M28" s="1"/>
       <c r="N28" s="1">
         <v>0</v>
       </c>
       <c r="O28" s="1">
-        <v>141750</v>
+        <v>63478</v>
       </c>
       <c r="P28" s="1">
-        <v>141750</v>
+        <v>158695</v>
       </c>
       <c r="Q28" t="s">
-        <v>108</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -5075,50 +5077,48 @@
         <v>201</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="C29" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="F29" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G29" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="H29" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I29" s="1">
-        <v>99984</v>
+        <v>136750</v>
       </c>
       <c r="J29" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="K29" s="1">
         <v>0</v>
       </c>
       <c r="L29" s="1"/>
-      <c r="M29" s="1">
-        <v>500</v>
-      </c>
+      <c r="M29" s="1"/>
       <c r="N29" s="1">
         <v>0</v>
       </c>
       <c r="O29" s="1">
-        <v>100484</v>
+        <v>141750</v>
       </c>
       <c r="P29" s="1">
-        <v>251210</v>
+        <v>141750</v>
       </c>
       <c r="Q29" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
@@ -5126,19 +5126,19 @@
         <v>202</v>
       </c>
       <c r="B30" t="s">
-        <v>154</v>
+        <v>80</v>
       </c>
       <c r="C30" t="s">
         <v>44</v>
       </c>
       <c r="D30" t="s">
-        <v>153</v>
+        <v>79</v>
       </c>
       <c r="E30" t="s">
         <v>32</v>
       </c>
       <c r="F30" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G30" t="s">
         <v>31</v>
@@ -5147,7 +5147,7 @@
         <v>35</v>
       </c>
       <c r="I30" s="1">
-        <v>107681</v>
+        <v>99984</v>
       </c>
       <c r="J30" s="1">
         <v>0</v>
@@ -5156,18 +5156,20 @@
         <v>0</v>
       </c>
       <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
+      <c r="M30" s="1">
+        <v>500</v>
+      </c>
       <c r="N30" s="1">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="O30" s="1">
-        <v>122681</v>
+        <v>100484</v>
       </c>
       <c r="P30" s="1">
-        <v>219980</v>
+        <v>251210</v>
       </c>
       <c r="Q30" t="s">
-        <v>155</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
@@ -5175,44 +5177,48 @@
         <v>203</v>
       </c>
       <c r="B31" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="C31" t="s">
-        <v>133</v>
+        <v>44</v>
       </c>
       <c r="D31" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="E31" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F31" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G31" t="s">
-        <v>103</v>
+        <v>31</v>
       </c>
       <c r="H31" t="s">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="I31" s="1">
-        <v>195000</v>
-      </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
+        <v>107681</v>
+      </c>
+      <c r="J31" s="1">
+        <v>0</v>
+      </c>
+      <c r="K31" s="1">
+        <v>0</v>
+      </c>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="O31" s="1">
-        <v>195000</v>
+        <v>122681</v>
       </c>
       <c r="P31" s="1">
-        <v>195000</v>
+        <v>219980</v>
       </c>
       <c r="Q31" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
@@ -5220,13 +5226,13 @@
         <v>204</v>
       </c>
       <c r="B32" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="C32" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="D32" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="E32" t="s">
         <v>24</v>
@@ -5235,35 +5241,29 @@
         <v>25</v>
       </c>
       <c r="G32" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H32" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="I32" s="1">
-        <v>157891</v>
-      </c>
-      <c r="J32" s="1">
-        <v>5500</v>
-      </c>
-      <c r="K32" s="1">
-        <v>0</v>
-      </c>
-      <c r="L32" s="1">
-        <v>1200</v>
-      </c>
+        <v>195000</v>
+      </c>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1">
         <v>0</v>
       </c>
       <c r="O32" s="1">
-        <v>164591</v>
+        <v>195000</v>
       </c>
       <c r="P32" s="1">
-        <v>164591</v>
+        <v>195000</v>
       </c>
       <c r="Q32" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
@@ -5271,50 +5271,50 @@
         <v>205</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="C33" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="D33" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="E33" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="F33" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="G33" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="H33" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="I33" s="1">
-        <v>57571</v>
+        <v>157891</v>
       </c>
       <c r="J33" s="1">
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="K33" s="1">
         <v>0</v>
       </c>
       <c r="L33" s="1">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="M33" s="1"/>
       <c r="N33" s="1">
         <v>0</v>
       </c>
       <c r="O33" s="1">
-        <v>57571</v>
+        <v>164591</v>
       </c>
       <c r="P33" s="1">
-        <v>146866</v>
+        <v>164591</v>
       </c>
       <c r="Q33" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
@@ -5328,19 +5328,19 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
+        <v>111</v>
+      </c>
+      <c r="E34" t="s">
+        <v>71</v>
+      </c>
+      <c r="F34" t="s">
         <v>113</v>
       </c>
-      <c r="E34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F34" t="s">
-        <v>73</v>
-      </c>
       <c r="G34" t="s">
-        <v>71</v>
+        <v>112</v>
       </c>
       <c r="H34" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="I34" s="1">
         <v>57219</v>

</xml_diff>

<commit_message>
Superintendent-pay: add Union as fourth reference contract + research memo
Union town clerk supplied the combined superintendent/principal
contracts (2025-2028 and successor 2026-2029). The supe role is a
$10,701 addendum to the $128,419 principal salary with no stated hours
split, so a research memo (research/union-combined-position/)
reconstructs the FTE-equivalent rate via the AASA supe:principal ratio
method: ~$210K-$230K, implied supe time ~5.5%. Treated reference-only,
parallel to Chaplin/RD 11. Pending districts drop from 5 to 4; contracts
subpage/zip/xlsx regenerated with the Union PDF.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/aes/superintendent-pay/contracts.xlsx
+++ b/reports/aes/superintendent-pay/contracts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="212">
   <si>
     <t>District</t>
   </si>
@@ -512,6 +512,18 @@
     <t>storrs/Morell_Mansfield_2025-2028.pdf</t>
   </si>
   <si>
+    <t>Union</t>
+  </si>
+  <si>
+    <t>Steven J. Jackopsic</t>
+  </si>
+  <si>
+    <t>PreK-8 (combined superintendent + elementary principal, one school; SpEd service administration PreK-12)</t>
+  </si>
+  <si>
+    <t>union/20260715114107674.pdf</t>
+  </si>
+  <si>
     <t>Slug</t>
   </si>
   <si>
@@ -555,6 +567,9 @@
   </si>
   <si>
     <t>amity-region-5</t>
+  </si>
+  <si>
+    <t>union</t>
   </si>
   <si>
     <t>hebron</t>
@@ -1023,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3613,6 +3628,64 @@
       </c>
       <c r="T44" t="s">
         <v>165</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>166</v>
+      </c>
+      <c r="B45" t="s">
+        <v>167</v>
+      </c>
+      <c r="C45" t="s">
+        <v>168</v>
+      </c>
+      <c r="D45" t="s">
+        <v>23</v>
+      </c>
+      <c r="E45" t="s">
+        <v>45</v>
+      </c>
+      <c r="F45" t="s">
+        <v>40</v>
+      </c>
+      <c r="G45">
+        <v>0.0547</v>
+      </c>
+      <c r="H45">
+        <v>0.0547</v>
+      </c>
+      <c r="I45" s="1">
+        <v>10701</v>
+      </c>
+      <c r="J45" s="1">
+        <v>1150</v>
+      </c>
+      <c r="K45" s="1">
+        <v>0</v>
+      </c>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1">
+        <v>800</v>
+      </c>
+      <c r="O45" s="1">
+        <v>12651</v>
+      </c>
+      <c r="P45" s="1">
+        <v>231273</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>34</v>
+      </c>
+      <c r="R45" t="s">
+        <v>27</v>
+      </c>
+      <c r="S45" t="s">
+        <v>28</v>
+      </c>
+      <c r="T45" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -3659,6 +3732,7 @@
     <hyperlink ref="T42" r:id="rId39"/>
     <hyperlink ref="T43" r:id="rId40"/>
     <hyperlink ref="T44" r:id="rId41"/>
+    <hyperlink ref="T45" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3667,7 +3741,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3684,7 +3758,7 @@
   <sheetData>
     <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -3693,16 +3767,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>17</v>
@@ -3737,7 +3811,7 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B2" t="s">
         <v>66</v>
@@ -3746,7 +3820,7 @@
         <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E2" t="s">
         <v>48</v>
@@ -3788,7 +3862,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
         <v>55</v>
@@ -3797,7 +3871,7 @@
         <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E3" t="s">
         <v>45</v>
@@ -3837,7 +3911,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B4" t="s">
         <v>38</v>
@@ -3886,7 +3960,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B5" t="s">
         <v>126</v>
@@ -3937,7 +4011,7 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B6" t="s">
         <v>136</v>
@@ -3946,7 +4020,7 @@
         <v>137</v>
       </c>
       <c r="D6" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E6" t="s">
         <v>45</v>
@@ -3986,7 +4060,7 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B7" t="s">
         <v>148</v>
@@ -4035,7 +4109,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B8" t="s">
         <v>119</v>
@@ -4086,16 +4160,16 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>167</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>168</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>166</v>
       </c>
       <c r="E9" t="s">
         <v>45</v>
@@ -4110,45 +4184,47 @@
         <v>27</v>
       </c>
       <c r="I9" s="1">
-        <v>213082</v>
+        <v>10701</v>
       </c>
       <c r="J9" s="1">
-        <v>10654.1</v>
-      </c>
-      <c r="K9" s="1"/>
+        <v>1150</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="O9" s="1">
-        <v>223736.1</v>
+        <v>12651</v>
       </c>
       <c r="P9" s="1">
-        <v>223736</v>
+        <v>231273</v>
       </c>
       <c r="Q9" t="s">
-        <v>78</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B10" t="s">
-        <v>145</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>144</v>
+        <v>76</v>
       </c>
       <c r="E10" t="s">
         <v>45</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G10" t="s">
         <v>23</v>
@@ -4157,56 +4233,54 @@
         <v>27</v>
       </c>
       <c r="I10" s="1">
-        <v>100000</v>
+        <v>213082</v>
       </c>
       <c r="J10" s="1">
-        <v>0</v>
-      </c>
-      <c r="K10" s="1">
-        <v>0</v>
-      </c>
+        <v>10654.1</v>
+      </c>
+      <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1">
         <v>0</v>
       </c>
       <c r="O10" s="1">
-        <v>100000</v>
+        <v>223736.1</v>
       </c>
       <c r="P10" s="1">
-        <v>222222</v>
+        <v>223736</v>
       </c>
       <c r="Q10" t="s">
-        <v>146</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>145</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>144</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F11" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="H11" t="s">
         <v>27</v>
       </c>
       <c r="I11" s="1">
-        <v>79552</v>
+        <v>100000</v>
       </c>
       <c r="J11" s="1">
         <v>0</v>
@@ -4214,90 +4288,90 @@
       <c r="K11" s="1">
         <v>0</v>
       </c>
-      <c r="L11" s="1">
-        <v>4000</v>
-      </c>
+      <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1">
         <v>0</v>
       </c>
       <c r="O11" s="1">
-        <v>83552</v>
+        <v>100000</v>
       </c>
       <c r="P11" s="1">
-        <v>208880</v>
+        <v>222222</v>
       </c>
       <c r="Q11" t="s">
-        <v>64</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="H12" t="s">
         <v>27</v>
       </c>
       <c r="I12" s="1">
-        <v>192400</v>
+        <v>79552</v>
       </c>
       <c r="J12" s="1">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K12" s="1">
         <v>0</v>
       </c>
-      <c r="L12" s="1"/>
+      <c r="L12" s="1">
+        <v>4000</v>
+      </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1">
         <v>0</v>
       </c>
       <c r="O12" s="1">
-        <v>202400</v>
+        <v>83552</v>
       </c>
       <c r="P12" s="1">
-        <v>202400</v>
+        <v>208880</v>
       </c>
       <c r="Q12" t="s">
-        <v>110</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B13" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="E13" t="s">
-        <v>45</v>
+        <v>109</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G13" t="s">
         <v>23</v>
@@ -4306,10 +4380,10 @@
         <v>27</v>
       </c>
       <c r="I13" s="1">
-        <v>80000</v>
+        <v>192400</v>
       </c>
       <c r="J13" s="1">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K13" s="1">
         <v>0</v>
@@ -4320,33 +4394,33 @@
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>80000</v>
+        <v>202400</v>
       </c>
       <c r="P13" s="1">
-        <v>200000</v>
+        <v>202400</v>
       </c>
       <c r="Q13" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B14" t="s">
-        <v>164</v>
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="D14" t="s">
-        <v>163</v>
+        <v>95</v>
       </c>
       <c r="E14" t="s">
         <v>45</v>
       </c>
       <c r="F14" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
         <v>23</v>
@@ -4355,10 +4429,10 @@
         <v>27</v>
       </c>
       <c r="I14" s="1">
-        <v>192000</v>
+        <v>80000</v>
       </c>
       <c r="J14" s="1">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="K14" s="1">
         <v>0</v>
@@ -4369,33 +4443,33 @@
         <v>0</v>
       </c>
       <c r="O14" s="1">
-        <v>200000</v>
+        <v>80000</v>
       </c>
       <c r="P14" s="1">
         <v>200000</v>
       </c>
       <c r="Q14" t="s">
-        <v>165</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>164</v>
       </c>
       <c r="C15" t="s">
         <v>44</v>
       </c>
       <c r="D15" t="s">
-        <v>115</v>
+        <v>163</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="G15" t="s">
         <v>23</v>
@@ -4404,10 +4478,10 @@
         <v>27</v>
       </c>
       <c r="I15" s="1">
-        <v>123739</v>
+        <v>192000</v>
       </c>
       <c r="J15" s="1">
-        <v>11650</v>
+        <v>8000</v>
       </c>
       <c r="K15" s="1">
         <v>0</v>
@@ -4415,36 +4489,36 @@
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>138389</v>
+        <v>200000</v>
       </c>
       <c r="P15" s="1">
-        <v>197699</v>
+        <v>200000</v>
       </c>
       <c r="Q15" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B16" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="D16" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="E16" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F16" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G16" t="s">
         <v>23</v>
@@ -4453,49 +4527,47 @@
         <v>27</v>
       </c>
       <c r="I16" s="1">
-        <v>75748</v>
+        <v>123739</v>
       </c>
       <c r="J16" s="1">
-        <v>0</v>
+        <v>11650</v>
       </c>
       <c r="K16" s="1">
         <v>0</v>
       </c>
-      <c r="L16" s="1">
-        <v>2500</v>
-      </c>
+      <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="O16" s="1">
-        <v>78248</v>
+        <v>138389</v>
       </c>
       <c r="P16" s="1">
-        <v>195620</v>
+        <v>197699</v>
       </c>
       <c r="Q16" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>82</v>
+        <v>128</v>
       </c>
       <c r="E17" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="F17" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G17" t="s">
         <v>23</v>
@@ -4504,10 +4576,10 @@
         <v>27</v>
       </c>
       <c r="I17" s="1">
-        <v>180250</v>
+        <v>75748</v>
       </c>
       <c r="J17" s="1">
-        <v>10500</v>
+        <v>0</v>
       </c>
       <c r="K17" s="1">
         <v>0</v>
@@ -4520,33 +4592,33 @@
         <v>0</v>
       </c>
       <c r="O17" s="1">
-        <v>193250</v>
+        <v>78248</v>
       </c>
       <c r="P17" s="1">
-        <v>193250</v>
+        <v>195620</v>
       </c>
       <c r="Q17" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B18" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="F18" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
         <v>23</v>
@@ -4555,47 +4627,49 @@
         <v>27</v>
       </c>
       <c r="I18" s="1">
-        <v>190000</v>
+        <v>180250</v>
       </c>
       <c r="J18" s="1">
-        <v>0</v>
+        <v>10500</v>
       </c>
       <c r="K18" s="1">
         <v>0</v>
       </c>
-      <c r="L18" s="1"/>
+      <c r="L18" s="1">
+        <v>2500</v>
+      </c>
       <c r="M18" s="1"/>
       <c r="N18" s="1">
         <v>0</v>
       </c>
       <c r="O18" s="1">
-        <v>190000</v>
+        <v>193250</v>
       </c>
       <c r="P18" s="1">
-        <v>190000</v>
+        <v>193250</v>
       </c>
       <c r="Q18" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B19" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C19" t="s">
         <v>44</v>
       </c>
       <c r="D19" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E19" t="s">
-        <v>158</v>
+        <v>45</v>
       </c>
       <c r="F19" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="G19" t="s">
         <v>23</v>
@@ -4604,10 +4678,10 @@
         <v>27</v>
       </c>
       <c r="I19" s="1">
-        <v>178190</v>
+        <v>190000</v>
       </c>
       <c r="J19" s="1">
-        <v>8910</v>
+        <v>0</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
@@ -4615,33 +4689,33 @@
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="O19" s="1">
-        <v>189100</v>
+        <v>190000</v>
       </c>
       <c r="P19" s="1">
-        <v>189100</v>
+        <v>190000</v>
       </c>
       <c r="Q19" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>157</v>
       </c>
       <c r="C20" t="s">
         <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>46</v>
+        <v>156</v>
       </c>
       <c r="E20" t="s">
-        <v>48</v>
+        <v>158</v>
       </c>
       <c r="F20" t="s">
         <v>49</v>
@@ -4653,10 +4727,10 @@
         <v>27</v>
       </c>
       <c r="I20" s="1">
-        <v>175000</v>
+        <v>178190</v>
       </c>
       <c r="J20" s="1">
-        <v>10000</v>
+        <v>8910</v>
       </c>
       <c r="K20" s="1">
         <v>0</v>
@@ -4664,30 +4738,30 @@
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="O20" s="1">
-        <v>185000</v>
+        <v>189100</v>
       </c>
       <c r="P20" s="1">
-        <v>185000</v>
+        <v>189100</v>
       </c>
       <c r="Q20" t="s">
-        <v>50</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B21" t="s">
-        <v>123</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="D21" t="s">
-        <v>122</v>
+        <v>46</v>
       </c>
       <c r="E21" t="s">
         <v>48</v>
@@ -4696,16 +4770,16 @@
         <v>49</v>
       </c>
       <c r="G21" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="H21" t="s">
         <v>27</v>
       </c>
       <c r="I21" s="1">
-        <v>177642.4</v>
+        <v>175000</v>
       </c>
       <c r="J21" s="1">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="K21" s="1">
         <v>0</v>
@@ -4716,27 +4790,27 @@
         <v>0</v>
       </c>
       <c r="O21" s="1">
-        <v>184642.4</v>
+        <v>185000</v>
       </c>
       <c r="P21" s="1">
-        <v>184642</v>
+        <v>185000</v>
       </c>
       <c r="Q21" t="s">
-        <v>124</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>123</v>
       </c>
       <c r="C22" t="s">
         <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>122</v>
       </c>
       <c r="E22" t="s">
         <v>48</v>
@@ -4745,16 +4819,16 @@
         <v>49</v>
       </c>
       <c r="G22" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="H22" t="s">
         <v>27</v>
       </c>
       <c r="I22" s="1">
-        <v>178448</v>
+        <v>177642.4</v>
       </c>
       <c r="J22" s="1">
-        <v>5353</v>
+        <v>7000</v>
       </c>
       <c r="K22" s="1">
         <v>0</v>
@@ -4765,33 +4839,33 @@
         <v>0</v>
       </c>
       <c r="O22" s="1">
-        <v>183801</v>
+        <v>184642.4</v>
       </c>
       <c r="P22" s="1">
-        <v>183801</v>
+        <v>184642</v>
       </c>
       <c r="Q22" t="s">
-        <v>53</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="E23" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F23" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G23" t="s">
         <v>23</v>
@@ -4800,10 +4874,10 @@
         <v>27</v>
       </c>
       <c r="I23" s="1">
-        <v>161690</v>
+        <v>178448</v>
       </c>
       <c r="J23" s="1">
-        <v>17617</v>
+        <v>5353</v>
       </c>
       <c r="K23" s="1">
         <v>0</v>
@@ -4814,27 +4888,27 @@
         <v>0</v>
       </c>
       <c r="O23" s="1">
-        <v>179307</v>
+        <v>183801</v>
       </c>
       <c r="P23" s="1">
-        <v>179307</v>
+        <v>183801</v>
       </c>
       <c r="Q23" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="D24" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="E24" t="s">
         <v>45</v>
@@ -4849,10 +4923,10 @@
         <v>27</v>
       </c>
       <c r="I24" s="1">
-        <v>53750</v>
+        <v>161690</v>
       </c>
       <c r="J24" s="1">
-        <v>0</v>
+        <v>17617</v>
       </c>
       <c r="K24" s="1">
         <v>0</v>
@@ -4863,33 +4937,33 @@
         <v>0</v>
       </c>
       <c r="O24" s="1">
-        <v>53750</v>
+        <v>179307</v>
       </c>
       <c r="P24" s="1">
-        <v>179167</v>
+        <v>179307</v>
       </c>
       <c r="Q24" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B25" t="s">
-        <v>151</v>
+        <v>74</v>
       </c>
       <c r="C25" t="s">
         <v>44</v>
       </c>
       <c r="D25" t="s">
-        <v>150</v>
+        <v>73</v>
       </c>
       <c r="E25" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="G25" t="s">
         <v>23</v>
@@ -4898,10 +4972,10 @@
         <v>27</v>
       </c>
       <c r="I25" s="1">
-        <v>75000</v>
+        <v>53750</v>
       </c>
       <c r="J25" s="1">
-        <v>2600</v>
+        <v>0</v>
       </c>
       <c r="K25" s="1">
         <v>0</v>
@@ -4912,133 +4986,133 @@
         <v>0</v>
       </c>
       <c r="O25" s="1">
-        <v>77600</v>
+        <v>53750</v>
       </c>
       <c r="P25" s="1">
-        <v>175443</v>
+        <v>179167</v>
       </c>
       <c r="Q25" t="s">
-        <v>152</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>151</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>150</v>
       </c>
       <c r="E26" t="s">
-        <v>87</v>
+        <v>48</v>
       </c>
       <c r="F26" t="s">
-        <v>88</v>
+        <v>49</v>
       </c>
       <c r="G26" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="H26" t="s">
         <v>27</v>
       </c>
       <c r="I26" s="1">
-        <v>63500</v>
+        <v>75000</v>
       </c>
       <c r="J26" s="1">
-        <v>0</v>
+        <v>2600</v>
       </c>
       <c r="K26" s="1">
         <v>0</v>
       </c>
-      <c r="L26" s="1">
-        <v>6000</v>
-      </c>
+      <c r="L26" s="1"/>
       <c r="M26" s="1"/>
       <c r="N26" s="1">
         <v>0</v>
       </c>
       <c r="O26" s="1">
-        <v>69500</v>
+        <v>77600</v>
       </c>
       <c r="P26" s="1">
-        <v>173750</v>
+        <v>175443</v>
       </c>
       <c r="Q26" t="s">
-        <v>89</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B27" t="s">
-        <v>21</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="E27" t="s">
-        <v>24</v>
+        <v>87</v>
       </c>
       <c r="F27" t="s">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="G27" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="H27" t="s">
         <v>27</v>
       </c>
       <c r="I27" s="1">
-        <v>90000</v>
+        <v>63500</v>
       </c>
       <c r="J27" s="1">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K27" s="1">
         <v>0</v>
       </c>
-      <c r="L27" s="1"/>
+      <c r="L27" s="1">
+        <v>6000</v>
+      </c>
       <c r="M27" s="1"/>
       <c r="N27" s="1">
         <v>0</v>
       </c>
       <c r="O27" s="1">
-        <v>100000</v>
+        <v>69500</v>
       </c>
       <c r="P27" s="1">
-        <v>166667</v>
+        <v>173750</v>
       </c>
       <c r="Q27" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B28" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="F28" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="G28" t="s">
         <v>23</v>
@@ -5047,46 +5121,44 @@
         <v>27</v>
       </c>
       <c r="I28" s="1">
-        <v>63478</v>
+        <v>90000</v>
       </c>
       <c r="J28" s="1">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K28" s="1">
         <v>0</v>
       </c>
-      <c r="L28" s="1">
-        <v>0</v>
-      </c>
+      <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1">
         <v>0</v>
       </c>
       <c r="O28" s="1">
-        <v>63478</v>
+        <v>100000</v>
       </c>
       <c r="P28" s="1">
-        <v>158695</v>
+        <v>166667</v>
       </c>
       <c r="Q28" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="F29" t="s">
         <v>49</v>
@@ -5098,98 +5170,98 @@
         <v>27</v>
       </c>
       <c r="I29" s="1">
-        <v>136750</v>
+        <v>63478</v>
       </c>
       <c r="J29" s="1">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="K29" s="1">
         <v>0</v>
       </c>
-      <c r="L29" s="1"/>
+      <c r="L29" s="1">
+        <v>0</v>
+      </c>
       <c r="M29" s="1"/>
       <c r="N29" s="1">
         <v>0</v>
       </c>
       <c r="O29" s="1">
-        <v>141750</v>
+        <v>63478</v>
       </c>
       <c r="P29" s="1">
-        <v>141750</v>
+        <v>158695</v>
       </c>
       <c r="Q29" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B30" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C30" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="D30" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="E30" t="s">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="F30" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G30" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="H30" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I30" s="1">
-        <v>99984</v>
+        <v>136750</v>
       </c>
       <c r="J30" s="1">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="K30" s="1">
         <v>0</v>
       </c>
       <c r="L30" s="1"/>
-      <c r="M30" s="1">
-        <v>500</v>
-      </c>
+      <c r="M30" s="1"/>
       <c r="N30" s="1">
         <v>0</v>
       </c>
       <c r="O30" s="1">
-        <v>100484</v>
+        <v>141750</v>
       </c>
       <c r="P30" s="1">
-        <v>251210</v>
+        <v>141750</v>
       </c>
       <c r="Q30" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B31" t="s">
-        <v>154</v>
+        <v>80</v>
       </c>
       <c r="C31" t="s">
         <v>44</v>
       </c>
       <c r="D31" t="s">
-        <v>153</v>
+        <v>79</v>
       </c>
       <c r="E31" t="s">
         <v>32</v>
       </c>
       <c r="F31" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G31" t="s">
         <v>31</v>
@@ -5198,7 +5270,7 @@
         <v>35</v>
       </c>
       <c r="I31" s="1">
-        <v>107681</v>
+        <v>99984</v>
       </c>
       <c r="J31" s="1">
         <v>0</v>
@@ -5207,77 +5279,83 @@
         <v>0</v>
       </c>
       <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
+      <c r="M31" s="1">
+        <v>500</v>
+      </c>
       <c r="N31" s="1">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="O31" s="1">
-        <v>122681</v>
+        <v>100484</v>
       </c>
       <c r="P31" s="1">
-        <v>219980</v>
+        <v>251210</v>
       </c>
       <c r="Q31" t="s">
-        <v>155</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B32" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="C32" t="s">
-        <v>133</v>
+        <v>44</v>
       </c>
       <c r="D32" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="E32" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F32" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G32" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="H32" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="I32" s="1">
-        <v>195000</v>
-      </c>
-      <c r="J32" s="1"/>
-      <c r="K32" s="1"/>
+        <v>107681</v>
+      </c>
+      <c r="J32" s="1">
+        <v>0</v>
+      </c>
+      <c r="K32" s="1">
+        <v>0</v>
+      </c>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="O32" s="1">
-        <v>195000</v>
+        <v>122681</v>
       </c>
       <c r="P32" s="1">
-        <v>195000</v>
+        <v>219980</v>
       </c>
       <c r="Q32" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B33" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="C33" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="D33" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
         <v>24</v>
@@ -5292,77 +5370,122 @@
         <v>101</v>
       </c>
       <c r="I33" s="1">
-        <v>157891</v>
-      </c>
-      <c r="J33" s="1">
-        <v>5500</v>
-      </c>
-      <c r="K33" s="1">
-        <v>0</v>
-      </c>
-      <c r="L33" s="1">
-        <v>1200</v>
-      </c>
+        <v>195000</v>
+      </c>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
       <c r="M33" s="1"/>
       <c r="N33" s="1">
         <v>0</v>
       </c>
       <c r="O33" s="1">
-        <v>164591</v>
+        <v>195000</v>
       </c>
       <c r="P33" s="1">
-        <v>164591</v>
+        <v>195000</v>
       </c>
       <c r="Q33" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B34" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="C34" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="D34" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="E34" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="F34" t="s">
-        <v>113</v>
+        <v>25</v>
       </c>
       <c r="G34" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="H34" t="s">
         <v>101</v>
       </c>
       <c r="I34" s="1">
-        <v>57219</v>
+        <v>157891</v>
       </c>
       <c r="J34" s="1">
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="K34" s="1">
         <v>0</v>
       </c>
-      <c r="L34" s="1"/>
+      <c r="L34" s="1">
+        <v>1200</v>
+      </c>
       <c r="M34" s="1"/>
       <c r="N34" s="1">
         <v>0</v>
       </c>
       <c r="O34" s="1">
+        <v>164591</v>
+      </c>
+      <c r="P34" s="1">
+        <v>164591</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>211</v>
+      </c>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35" t="s">
+        <v>111</v>
+      </c>
+      <c r="E35" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" t="s">
+        <v>113</v>
+      </c>
+      <c r="G35" t="s">
+        <v>112</v>
+      </c>
+      <c r="H35" t="s">
+        <v>101</v>
+      </c>
+      <c r="I35" s="1">
         <v>57219</v>
       </c>
-      <c r="P34" s="1">
+      <c r="J35" s="1">
+        <v>0</v>
+      </c>
+      <c r="K35" s="1">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1">
+        <v>0</v>
+      </c>
+      <c r="O35" s="1">
+        <v>57219</v>
+      </c>
+      <c r="P35" s="1">
         <v>143048</v>
       </c>
-      <c r="Q34" t="s">
+      <c r="Q35" t="s">
         <v>114</v>
       </c>
     </row>
@@ -5402,6 +5525,7 @@
     <hyperlink ref="Q32" r:id="rId31"/>
     <hyperlink ref="Q33" r:id="rId32"/>
     <hyperlink ref="Q34" r:id="rId33"/>
+    <hyperlink ref="Q35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>